<commit_message>
feat: Macaulay Library taxonCode を学名から取得しExcelに追加
248/258種の taxonCode を taxonomy API で自動取得。
10種は ML 未登録のため空欄。

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/animal-sounds-data.xlsx
+++ b/data/animal-sounds-data.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="メインデータ" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="名称マッピング" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分類マッピング" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="オノマトペマッピング" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="凡例・定義" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地域マスター" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地域マッピング" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="メインデータ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="名称マッピング" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="分類マッピング" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="オノマトペマッピング" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="凡例・定義" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="地域マスター" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="地域マッピング" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'メインデータ'!$A$1:$M$248</definedName>
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N259"/>
+  <dimension ref="A1:O259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -605,6 +605,11 @@
           <t>音声参照</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>taxonCode</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -673,6 +678,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Macaca%20fuscata</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>t-12077600</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -741,6 +751,11 @@
           <t>https://xeno-canto.org/species/Corvus-macrorhynchos</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>labcro1</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -809,6 +824,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Dryophytes%20japonicus</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>t-11039482</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -875,6 +895,11 @@
       <c r="N5" t="inlineStr">
         <is>
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Teleogryllus%20emma</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>t-12137860</t>
         </is>
       </c>
     </row>
@@ -941,6 +966,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Caretta%20caretta</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>t-12104433</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1009,6 +1039,11 @@
           <t>https://xeno-canto.org/species/Passer-montanus</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>eutspa</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1081,6 +1116,11 @@
           <t>https://xeno-canto.org/species/Corvus-corone</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>carcro1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1153,6 +1193,11 @@
           <t>https://xeno-canto.org/species/Horornis-diphone</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>jabwar</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1221,6 +1266,11 @@
           <t>https://xeno-canto.org/species/Zosterops-japonicus</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>warwhe1</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1293,6 +1343,11 @@
           <t>https://xeno-canto.org/species/Parus-minor</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>japtit4</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1361,6 +1416,11 @@
           <t>https://xeno-canto.org/species/Sittiparus-varius</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>vartit1</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1433,6 +1493,11 @@
           <t>https://xeno-canto.org/species/Alauda-arvensis</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>skylar</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1501,6 +1566,11 @@
           <t>https://xeno-canto.org/species/Hirundo-rustica</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>barswa</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1573,6 +1643,11 @@
           <t>https://xeno-canto.org/species/Cyanoptila-cyanomelana</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>bawfly2</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1645,6 +1720,11 @@
           <t>https://xeno-canto.org/species/Larvivora-akahige</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>japrob2</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1717,6 +1797,11 @@
           <t>https://xeno-canto.org/species/Phoenicurus-auroreus</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>daured1</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1789,6 +1874,11 @@
           <t>https://xeno-canto.org/species/Lanius-bucephalus</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>buhshr1</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1857,6 +1947,11 @@
           <t>https://xeno-canto.org/species/Motacilla-alba</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>whiwag</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1925,6 +2020,11 @@
           <t>https://xeno-canto.org/species/Chloris-sinica</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>origre</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1997,6 +2097,11 @@
           <t>https://xeno-canto.org/species/Emberiza-cioides</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>meabun1</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2069,6 +2174,11 @@
           <t>https://xeno-canto.org/species/Garrulus-glandarius</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>eurjay1</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2137,6 +2247,11 @@
           <t>https://xeno-canto.org/species/Cyanopica-cyanus</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>azwmag2</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2205,6 +2320,11 @@
           <t>https://xeno-canto.org/species/Hypsipetes-amaurotis</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>brebul1</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2273,6 +2393,11 @@
           <t>https://xeno-canto.org/species/Spodiopsar-cineraceus</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>whcsta1</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2341,6 +2466,11 @@
           <t>https://xeno-canto.org/species/Aegithalos-caudatus</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>lottit1</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2413,6 +2543,11 @@
           <t>https://xeno-canto.org/species/Alcedo-atthis</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>comkin1</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2485,6 +2620,11 @@
           <t>https://xeno-canto.org/species/Terpsiphone-atrocaudata</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>japfly1</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2557,6 +2697,11 @@
           <t>https://xeno-canto.org/species/Monticola-solitarius</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>burthr</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2629,6 +2774,11 @@
           <t>https://xeno-canto.org/species/Troglodytes-troglodytes</t>
         </is>
       </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>winwre4</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2701,6 +2851,11 @@
           <t>https://xeno-canto.org/species/Phasianus-versicolor</t>
         </is>
       </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>rinphe2</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2773,6 +2928,11 @@
           <t>https://xeno-canto.org/species/Syrmaticus-soemmerringii</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>copphe1</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2845,6 +3005,11 @@
           <t>https://xeno-canto.org/species/Lagopus-muta</t>
         </is>
       </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>rocpta1</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2917,6 +3082,11 @@
           <t>https://xeno-canto.org/species/Bambusicola-thoracicus</t>
         </is>
       </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>chbpar3</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2985,6 +3155,11 @@
           <t>https://xeno-canto.org/species/Coturnix-japonica</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>japqua</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3053,6 +3228,11 @@
           <t>https://xeno-canto.org/species/Anas-platyrhynchos</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>mallar3</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3121,6 +3301,11 @@
           <t>https://xeno-canto.org/species/Aix-galericulata</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>manduc</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3193,6 +3378,11 @@
           <t>https://xeno-canto.org/species/Cygnus-cygnus</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>whoswa</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3261,6 +3451,11 @@
           <t>https://xeno-canto.org/species/Anas-zonorhyncha</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>spbduc</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3333,6 +3528,11 @@
           <t>https://xeno-canto.org/species/Anas-crecca</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>gnwtea</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3401,6 +3601,11 @@
           <t>https://xeno-canto.org/species/Streptopelia-orientalis</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>ortdov</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3473,6 +3678,11 @@
           <t>https://xeno-canto.org/species/Columba-livia</t>
         </is>
       </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>rocpig</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3541,6 +3751,11 @@
           <t>https://xeno-canto.org/species/Treron-sieboldii</t>
         </is>
       </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>whbpig1</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3609,6 +3824,11 @@
           <t>https://xeno-canto.org/species/Accipiter-gentilis</t>
         </is>
       </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>y00392</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3677,6 +3897,11 @@
           <t>https://xeno-canto.org/species/Milvus-migrans</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>blakit1</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3745,6 +3970,11 @@
           <t>https://xeno-canto.org/species/Buteo-japonicus</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>combuz6</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3817,6 +4047,11 @@
           <t>https://xeno-canto.org/species/Haliaeetus-albicilla</t>
         </is>
       </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>whteag</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3889,6 +4124,11 @@
           <t>https://xeno-canto.org/species/Nisaetus-nipalensis</t>
         </is>
       </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>mouhae1</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3961,6 +4201,11 @@
           <t>https://xeno-canto.org/species/Strix-uralensis</t>
         </is>
       </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>uraowl1</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4029,6 +4274,11 @@
           <t>https://xeno-canto.org/species/Ninox-scutulata</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>brnhao1</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4101,6 +4351,11 @@
           <t>https://xeno-canto.org/species/Otus-scops</t>
         </is>
       </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>eursco1</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4173,6 +4428,11 @@
           <t>https://xeno-canto.org/species/Ketupa-blakistoni</t>
         </is>
       </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>blfowl1</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4245,6 +4505,11 @@
           <t>https://xeno-canto.org/species/Cuculus-canorus</t>
         </is>
       </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>comcuc</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4317,6 +4582,11 @@
           <t>https://xeno-canto.org/species/Cuculus-poliocephalus</t>
         </is>
       </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>lescuc1</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4389,6 +4659,11 @@
           <t>https://xeno-canto.org/species/Cuculus-optatus</t>
         </is>
       </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>oricuc2</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4461,6 +4736,11 @@
           <t>https://xeno-canto.org/species/Picus-awokera</t>
         </is>
       </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>japwoo1</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4529,6 +4809,11 @@
           <t>https://xeno-canto.org/species/Dendrocopos-major</t>
         </is>
       </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>grswoo</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4601,6 +4886,11 @@
           <t>https://xeno-canto.org/species/Yungipicus-kizuki</t>
         </is>
       </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>pygwoo1</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4669,6 +4959,11 @@
           <t>https://xeno-canto.org/species/Ardea-cinerea</t>
         </is>
       </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>graher1</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4737,6 +5032,11 @@
           <t>https://xeno-canto.org/species/Ardea-alba</t>
         </is>
       </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>greegr</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4809,6 +5109,11 @@
           <t>https://xeno-canto.org/species/Nycticorax-nycticorax</t>
         </is>
       </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>bcnher</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4881,6 +5186,11 @@
           <t>https://xeno-canto.org/species/Grus-japonensis</t>
         </is>
       </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>reccra1</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4953,6 +5263,11 @@
           <t>https://xeno-canto.org/species/Grus-monacha</t>
         </is>
       </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>hoocra1</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5021,6 +5336,11 @@
           <t>https://xeno-canto.org/species/Gallinula-chloropus</t>
         </is>
       </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>commoo3</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5093,6 +5413,11 @@
           <t>https://xeno-canto.org/species/Hypotaenidia-okinawae</t>
         </is>
       </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>okirai1</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5161,6 +5486,11 @@
           <t>https://xeno-canto.org/species/Chroicocephalus-ridibundus</t>
         </is>
       </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>bkhgul</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5233,6 +5563,11 @@
           <t>https://xeno-canto.org/species/Larus-crassirostris</t>
         </is>
       </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>bktgul</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5301,6 +5636,11 @@
           <t>https://xeno-canto.org/species/Charadrius-dubius</t>
         </is>
       </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>y00379</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5373,6 +5713,11 @@
           <t>https://xeno-canto.org/species/Gallinago-gallinago</t>
         </is>
       </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>comsni</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5445,6 +5790,11 @@
           <t>https://xeno-canto.org/species/Eurystomus-orientalis</t>
         </is>
       </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>dollar1</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5513,6 +5863,11 @@
           <t>https://xeno-canto.org/species/Megaceryle-lugubris</t>
         </is>
       </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>crekin1</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5585,6 +5940,11 @@
           <t>https://xeno-canto.org/species/Ciconia-boyciana</t>
         </is>
       </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>oristo1</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5653,6 +6013,11 @@
           <t>https://xeno-canto.org/species/Tachybaptus-ruficollis</t>
         </is>
       </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>litgre1</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5725,6 +6090,11 @@
           <t>https://xeno-canto.org/species/Calonectris-leucomelas</t>
         </is>
       </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>strshe</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5797,6 +6167,11 @@
           <t>https://xeno-canto.org/species/Aptenodytes-forsteri</t>
         </is>
       </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>emppen1</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5869,6 +6244,11 @@
           <t>https://xeno-canto.org/species/Upupa-epops</t>
         </is>
       </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>hoopoe</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5937,6 +6317,11 @@
           <t>https://xeno-canto.org/species/Apus-pacificus</t>
         </is>
       </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>fotswi</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6005,6 +6390,11 @@
           <t>https://xeno-canto.org/species/Gallus-gallus-domesticus</t>
         </is>
       </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>redjun1</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6073,6 +6463,11 @@
           <t>https://xeno-canto.org/species/Pavo-cristatus</t>
         </is>
       </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>compea</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -6145,6 +6540,11 @@
           <t>https://xeno-canto.org/species/Haliaeetus-leucocephalus</t>
         </is>
       </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>baleag</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6217,6 +6617,11 @@
           <t>https://xeno-canto.org/species/Menura-novaehollandiae</t>
         </is>
       </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>suplyr1</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6289,6 +6694,11 @@
           <t>https://xeno-canto.org/species/Luscinia-megarhynchos</t>
         </is>
       </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>comnig1</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6361,6 +6771,11 @@
           <t>https://xeno-canto.org/species/Apteryx-mantelli</t>
         </is>
       </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>nibkiw1</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6433,6 +6848,11 @@
           <t>https://xeno-canto.org/species/Dacelo-novaeguineae</t>
         </is>
       </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>laukoo1</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6505,6 +6925,11 @@
           <t>https://xeno-canto.org/species/Vultur-gryphus</t>
         </is>
       </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>andcon1</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6577,6 +7002,11 @@
           <t>https://xeno-canto.org/species/Phalacrocorax-capillatus</t>
         </is>
       </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>japcor1</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6649,6 +7079,11 @@
           <t>https://xeno-canto.org/species/Cinclus-pallasii</t>
         </is>
       </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>brodip1</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6717,6 +7152,11 @@
           <t>https://xeno-canto.org/species/Ficedula-narcissina</t>
         </is>
       </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>narfly2</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -6789,6 +7229,11 @@
           <t>https://xeno-canto.org/species/Pericrocotus-divaricatus</t>
         </is>
       </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>ashmin1</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6861,6 +7306,11 @@
           <t>https://xeno-canto.org/species/Phylloscopus-xanthodryas</t>
         </is>
       </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>arcwar3</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -6933,6 +7383,11 @@
           <t>https://xeno-canto.org/species/Phylloscopus-coronatus</t>
         </is>
       </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>eacwar1</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -7005,6 +7460,11 @@
           <t>https://xeno-canto.org/species/Acrocephalus-orientalis</t>
         </is>
       </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>orrwar1</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -7077,6 +7537,11 @@
           <t>https://xeno-canto.org/species/Nipponia-nippon</t>
         </is>
       </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>creibi1</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -7149,6 +7614,11 @@
           <t>https://xeno-canto.org/species/Anser-fabalis</t>
         </is>
       </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>taibeg1</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -7221,6 +7691,11 @@
           <t>https://xeno-canto.org/species/Gavia-stellata</t>
         </is>
       </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>retloo</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -7293,6 +7768,11 @@
           <t>https://xeno-canto.org/species/Struthio-camelus</t>
         </is>
       </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>ostric2</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -7361,6 +7841,11 @@
           <t>https://xeno-canto.org/species/Melopsittacus-undulatus</t>
         </is>
       </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>budger</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -7429,6 +7914,11 @@
           <t>https://xeno-canto.org/species/Nymphicus-hollandicus</t>
         </is>
       </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>cockat</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -7497,6 +7987,11 @@
           <t>https://xeno-canto.org/species/Phoenicopterus-roseus</t>
         </is>
       </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>grefla3</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -7637,6 +8132,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Felis%20catus</t>
         </is>
       </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>t-11031969</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -7705,6 +8205,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Panthera%20leo</t>
         </is>
       </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>t-11031947</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -7773,6 +8278,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Panthera%20tigris</t>
         </is>
       </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>t-11036143</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -7841,6 +8351,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Canis%20lupus</t>
         </is>
       </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>t-11032766</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -7909,6 +8424,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Vulpes%20vulpes%20japonica</t>
         </is>
       </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>t-12082798</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -7981,6 +8501,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Nyctereutes%20procyonoides</t>
         </is>
       </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>t-12084019</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -8049,6 +8574,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Ursus%20thibetanus</t>
         </is>
       </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>t-12076666</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -8121,6 +8651,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Ursus%20arctos</t>
         </is>
       </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>t-11038647</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -8189,6 +8724,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Ursus%20maritimus</t>
         </is>
       </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>t-11030301</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -8257,6 +8797,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Ailuropoda%20melanoleuca</t>
         </is>
       </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>t-12076675</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -8329,6 +8874,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Lutra%20nippon</t>
         </is>
       </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>t-12084968</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -8397,6 +8947,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Enhydra%20lutris</t>
         </is>
       </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>t-11036138</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -8465,6 +9020,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Phoca%20largha</t>
         </is>
       </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>t-11032768</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -8533,6 +9093,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Zalophus%20japonicus</t>
         </is>
       </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>t-12076704</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -8601,6 +9166,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Odobenus%20rosmarus</t>
         </is>
       </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>t-11030303</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -8669,6 +9239,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Crocuta%20crocuta</t>
         </is>
       </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>t-11074122</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -8741,6 +9316,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Acinonyx%20jubatus</t>
         </is>
       </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>t-11026957</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -8809,6 +9389,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Procyon%20lotor</t>
         </is>
       </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>t-11037790</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -8877,6 +9462,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Martes%20melampus</t>
         </is>
       </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>t-12076724</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -8945,6 +9535,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Bos%20taurus</t>
         </is>
       </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>t-11072529</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -9013,6 +9608,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Ovis%20aries</t>
         </is>
       </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>t-11067775</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -9081,6 +9681,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Capra%20aegagrus%20hircus</t>
         </is>
       </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>t-11076487</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -9149,6 +9754,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Sus%20scrofa%20domesticus</t>
         </is>
       </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>t-12041182</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -9217,6 +9827,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Sus%20scrofa</t>
         </is>
       </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>t-11074908</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -9289,6 +9904,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Cervus%20nippon</t>
         </is>
       </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>t-11078085</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -9357,6 +9977,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Rangifer%20tarandus</t>
         </is>
       </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>t-11070148</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -9429,6 +10054,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Capricornis%20crispus</t>
         </is>
       </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>t-12080269</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -9501,6 +10131,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Giraffa%20camelopardalis</t>
         </is>
       </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>t-11070143</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -9569,6 +10204,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Hippopotamus%20amphibius</t>
         </is>
       </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>t-11066977</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -9641,6 +10281,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Megaptera%20novaeangliae</t>
         </is>
       </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>t-11028617</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -9709,6 +10354,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Physeter%20macrocephalus</t>
         </is>
       </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>t-1474677</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -9777,6 +10427,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Orcinus%20orca</t>
         </is>
       </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>t-11038646</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -9845,6 +10500,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Tursiops%20truncatus</t>
         </is>
       </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>t-11033635</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -9913,6 +10573,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Camelus%20dromedarius</t>
         </is>
       </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>t-11066978</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -9981,6 +10646,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Vicugna%20pacos</t>
         </is>
       </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>t-12081106</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -10049,6 +10719,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Equus%20caballus</t>
         </is>
       </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>t-12030474</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -10117,6 +10792,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Equus%20asinus</t>
         </is>
       </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>t-12030473</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -10189,6 +10869,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Equus%20quagga</t>
         </is>
       </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>t-11069346</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -10257,6 +10942,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Ceratotherium%20simum</t>
         </is>
       </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>t-12077570</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -10325,6 +11015,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Loxodonta%20africana</t>
         </is>
       </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>t-11075812</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -10393,6 +11088,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Elephas%20maximus</t>
         </is>
       </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>t-11075768</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -10461,6 +11161,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Pan%20troglodytes</t>
         </is>
       </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>t-11062382</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -10529,6 +11234,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Gorilla%20gorilla</t>
         </is>
       </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>t-11064823</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -10597,6 +11307,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Hylobates%20lar</t>
         </is>
       </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>t-11053497</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -10665,6 +11380,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Alouatta%20seniculus</t>
         </is>
       </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>t-11057514</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -10733,6 +11453,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Lemur%20catta</t>
         </is>
       </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>t-11056709</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -10801,6 +11526,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Mus%20musculus</t>
         </is>
       </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>t-12078329</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -10869,6 +11599,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Rattus%20norvegicus</t>
         </is>
       </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>t-12078236</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -10937,6 +11672,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Sciurus%20lis</t>
         </is>
       </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>t-12079377</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -11009,6 +11749,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Petaurista%20leucogenys</t>
         </is>
       </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>t-12079370</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -11081,6 +11826,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Hydrochoerus%20hydrochaeris</t>
         </is>
       </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>t-11072558</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -11149,6 +11899,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Cavia%20porcellus</t>
         </is>
       </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>t-11076522</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -11217,6 +11972,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Mesocricetus%20auratus</t>
         </is>
       </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>t-12078507</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -11289,6 +12049,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Castor%20canadensis</t>
         </is>
       </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>t-11036119</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -11361,6 +12126,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Lepus%20brachyurus</t>
         </is>
       </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>t-12077436</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -11433,6 +12203,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Pentalagus%20furnessi</t>
         </is>
       </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>t-12077455</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -11505,6 +12280,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Ochotona%20hyperborea</t>
         </is>
       </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>t-12083931</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -11577,6 +12357,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Pteropus%20pselaphon</t>
         </is>
       </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>t-12076148</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -11649,6 +12434,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Pipistrellus%20abramus</t>
         </is>
       </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>t-12080850</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -11717,6 +12507,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Mogera%20imaizumii</t>
         </is>
       </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>t-12079953</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -11789,6 +12584,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Phascolarctos%20cinereus</t>
         </is>
       </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>t-11055109</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -11857,6 +12657,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Osphranter%20rufus</t>
         </is>
       </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>t-11063203</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -11925,6 +12730,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Sarcophilus%20harrisii</t>
         </is>
       </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>t-11046931</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -11993,6 +12803,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Orycteropus%20afer</t>
         </is>
       </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>t-12079982</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -12061,6 +12876,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Dasypus%20novemcinctus</t>
         </is>
       </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>t-11037804</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -12133,6 +12953,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Manis%20javanica</t>
         </is>
       </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>t-12077578</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -12205,6 +13030,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Meloimorpha%20japonica</t>
         </is>
       </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>t-12142599</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -12277,6 +13107,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Xenogryllus%20marmoratus</t>
         </is>
       </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>t-12141332</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -12349,6 +13184,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Velarifictorus%20micado</t>
         </is>
       </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>t-11870891</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -12417,6 +13257,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Loxoblemmus%20doenitzi</t>
         </is>
       </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>t-12156928</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -12489,6 +13334,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Oecanthus%20longicauda</t>
         </is>
       </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>t-12140054</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -12561,6 +13411,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Truljalia%20hibinonis</t>
         </is>
       </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>t-12134465</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -12633,6 +13488,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Ornebius%20kanetataki</t>
         </is>
       </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>t-12162519</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -12701,6 +13561,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Svistella%20bifasciata</t>
         </is>
       </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>t-12161659</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -12773,6 +13638,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Gampsocleis%20buergeri</t>
         </is>
       </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>t-12180976</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -12917,6 +13787,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Hexacentrus%20japonicus</t>
         </is>
       </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>t-12148298</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -13057,6 +13932,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Locusta%20migratoria</t>
         </is>
       </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>t-12119273</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -13129,6 +14009,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Acrida%20cinerea</t>
         </is>
       </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>t-12134456</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -13201,6 +14086,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Graptopsaltria%20nigrofuscata</t>
         </is>
       </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>t-12130907</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -13269,6 +14159,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Hyalessa%20maculaticollis</t>
         </is>
       </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>t-12134926</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -13341,6 +14236,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Cryptotympana%20facialis</t>
         </is>
       </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>t-12106542</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -13413,6 +14313,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Meimuna%20opalifera</t>
         </is>
       </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>t-12130764</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -13485,6 +14390,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Tanna%20japonensis</t>
         </is>
       </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>t-12134174</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -13773,6 +14683,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Apis%20mellifera</t>
         </is>
       </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>t-11139707</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -13841,6 +14756,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Apis%20cerana%20japonica</t>
         </is>
       </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>t-12931908</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -13913,6 +14833,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Vespa%20mandarinia</t>
         </is>
       </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>t-12918886</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -13985,6 +14910,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Aedes%20albopictus</t>
         </is>
       </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>t-12897703</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -14053,6 +14983,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Musca%20domestica</t>
         </is>
       </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>t-12906097</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -14125,6 +15060,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Trypoxylus%20dichotomus</t>
         </is>
       </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>t-12919021</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -14269,6 +15209,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Cephonodes%20hylas</t>
         </is>
       </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>t-12112331</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -14341,6 +15286,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Gromphadorhina%20portentosa</t>
         </is>
       </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>t-12918910</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -14413,6 +15363,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Anotogaster%20sieboldii</t>
         </is>
       </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>t-12105523</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -14481,6 +15436,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Pelophylax%20nigromaculatus</t>
         </is>
       </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>t-11102654</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -14553,6 +15513,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Lithobates%20catesbeianus</t>
         </is>
       </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>t-11113588</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -14697,6 +15662,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Zhangixalus%20arboreus</t>
         </is>
       </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>t-12094585</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -14769,6 +15739,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Zhangixalus%20schlegelii</t>
         </is>
       </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>t-12094587</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -14841,6 +15816,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Buergeria%20buergeri</t>
         </is>
       </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>t-12089661</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
@@ -14913,6 +15893,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Rana%20tagoi</t>
         </is>
       </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>t-12089325</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -14985,6 +15970,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Rana%20ornativentris</t>
         </is>
       </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>t-12089343</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -15053,6 +16043,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Rana%20japonica</t>
         </is>
       </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>t-12089322</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -15125,6 +16120,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Pelophylax%20porosus</t>
         </is>
       </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>t-12091381</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
@@ -15197,6 +16197,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Kurixalus%20eiffingeri</t>
         </is>
       </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>t-12089672</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -15269,6 +16274,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Odorrana%20ishikawae</t>
         </is>
       </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>t-12091322</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -15341,6 +16351,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Andrias%20japonicus</t>
         </is>
       </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>t-12089731</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -15409,6 +16424,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Cynops%20pyrrhogaster</t>
         </is>
       </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>t-12090190</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -15481,6 +16501,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Dendrobates%20tinctorius</t>
         </is>
       </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>t-12087506</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -15553,6 +16578,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Eleutherodactylus%20coqui</t>
         </is>
       </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>t-11130532</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
@@ -15625,6 +16655,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Xenopus%20laevis</t>
         </is>
       </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>t-12089309</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -15693,6 +16728,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Gekko%20japonicus</t>
         </is>
       </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>t-12108757</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -15765,6 +16805,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Gekko%20gecko</t>
         </is>
       </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>t-11774257</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -15837,6 +16882,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Elaphe%20climacophora</t>
         </is>
       </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>t-12105705</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -15909,6 +16959,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Gloydius%20blomhoffii</t>
         </is>
       </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>t-12098591</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -15981,6 +17036,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Crotalus%20atrox</t>
         </is>
       </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>t-11756105</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -16053,6 +17113,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Ophiophagus%20hannah</t>
         </is>
       </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>t-11770590</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -16125,6 +17190,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Crocodylus%20porosus</t>
         </is>
       </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>t-12096150</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -16193,6 +17263,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Alligator%20mississippiensis</t>
         </is>
       </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>t-11746735</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -16265,6 +17340,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Aldabrachelys%20gigantea</t>
         </is>
       </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>t-12030471</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -16337,6 +17417,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Pelodiscus%20sinensis</t>
         </is>
       </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>t-12105702</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -16407,6 +17492,11 @@
       <c r="N226" t="inlineStr">
         <is>
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Sphenodon%20punctatus</t>
+        </is>
+      </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>t-12119171</t>
         </is>
       </c>
     </row>
@@ -16473,6 +17563,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Plestiodon%20japonicus</t>
         </is>
       </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>t-12110377</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -16545,6 +17640,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Varanus%20komodoensis</t>
         </is>
       </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>t-12104272</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
@@ -16617,6 +17717,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Furcifer%20pardalis</t>
         </is>
       </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>t-12099735</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -16689,6 +17794,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Chelidonichthys%20spinosus</t>
         </is>
       </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>t-12921190</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
@@ -16761,6 +17871,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Oplegnathus%20fasciatus</t>
         </is>
       </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>t-12922796</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -16833,6 +17948,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Takifugu%20rubripes</t>
         </is>
       </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>t-12906043</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
@@ -16905,6 +18025,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Stephanolepis%20cirrhifer</t>
         </is>
       </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>t-12923047</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
@@ -16977,6 +18102,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Amphiprion%20ocellaris</t>
         </is>
       </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>t-12907675</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
@@ -17049,6 +18179,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Porichthys%20notatus</t>
         </is>
       </c>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>t-10857897</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -17121,6 +18256,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Nibea%20mitsukurii</t>
         </is>
       </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>t-12936257</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
@@ -17193,6 +18333,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Pygocentrus%20nattereri</t>
         </is>
       </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>pygnat1</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -17265,6 +18410,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Opsanus%20tau</t>
         </is>
       </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>t-10869486</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
@@ -17337,6 +18487,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Haemulon%20sciurus</t>
         </is>
       </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>t-10948810</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -17409,6 +18564,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Pagrus%20major</t>
         </is>
       </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>t-12907662</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
@@ -17477,6 +18637,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Sebastiscus%20marmoratus</t>
         </is>
       </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>t-12921074</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -17549,6 +18714,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Alpheus%20bellulus</t>
         </is>
       </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>t-12939602</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
@@ -17621,6 +18791,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Panulirus%20japonicus</t>
         </is>
       </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>t-12903755</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -17693,6 +18868,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Odontodactylus%20scyllarus</t>
         </is>
       </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>t-12906041</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
@@ -17765,6 +18945,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Ocypode%20stimpsoni</t>
         </is>
       </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>t-12461434</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
@@ -17837,6 +19022,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Homarus%20americanus</t>
         </is>
       </c>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>t-12897498</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
@@ -17909,6 +19099,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Mizuhopecten%20yessoensis</t>
         </is>
       </c>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>t-12919007</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -17976,6 +19171,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Buergeria%20buergeri</t>
         </is>
       </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>t-12089661</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -18043,6 +19243,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Hyla%20arborea</t>
         </is>
       </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>t-11156829</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -18110,6 +19315,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Hyla%20meridionalis</t>
         </is>
       </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>t-12088534</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -18177,6 +19387,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Dyscophus%20guineti</t>
         </is>
       </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>t-12089102</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -18244,6 +19459,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Cynops%20pyrrhogaster</t>
         </is>
       </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>t-12090190</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -18311,6 +19531,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Fejervarya%20kawamurai</t>
         </is>
       </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>t-12092612</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -18378,6 +19603,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Phyllobates%20aurotaenia</t>
         </is>
       </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>t-11145721</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -18445,6 +19675,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Rhinella%20marina</t>
         </is>
       </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>t-11147981</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -18574,6 +19809,11 @@
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Andrias%20davidianus</t>
         </is>
       </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>t-12089732</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -18701,6 +19941,11 @@
       <c r="N259" t="inlineStr">
         <is>
           <t>https://search.macaulaylibrary.org/catalog?taxonCode=&amp;mediaType=audio&amp;q=Microhyla%20ornata</t>
+        </is>
+      </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>t-11047001</t>
         </is>
       </c>
     </row>

</xml_diff>